<commit_message>
Fix spelling of coastal in farms.xlsx
</commit_message>
<xml_diff>
--- a/datascience/suitability_scoring/notebooks/temp_data/farms.xlsx
+++ b/datascience/suitability_scoring/notebooks/temp_data/farms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darrin\Work\Planting_Optimisation_tool_dws\datascience\suitability_scoring\notebooks\temp_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C735AE30-4093-407B-A6DB-D10FE367E26A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27956B13-68AF-456E-8061-2F5F007D106E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-285" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,10 +89,10 @@
     <t>longitude</t>
   </si>
   <si>
-    <t>costal</t>
+    <t>riparian</t>
   </si>
   <si>
-    <t>riparian</t>
+    <t>coastal</t>
   </si>
 </sst>
 </file>
@@ -398,10 +398,10 @@
         <v>16</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -33188,6 +33188,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="7998ff36-f67b-497d-9ba5-0737ce74e881" xsi:nil="true"/>
@@ -33202,15 +33211,6 @@
     <Axehead xmlns="5433951f-06c3-4618-8b57-3de8e57a9660" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -33233,6 +33233,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B6598FE-0BB4-48C7-B790-7641F110978B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9EEBAB-4FB8-43D1-946C-52B3C2DF27CE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -33241,12 +33249,4 @@
     <ds:schemaRef ds:uri="5433951f-06c3-4618-8b57-3de8e57a9660"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B6598FE-0BB4-48C7-B790-7641F110978B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>